<commit_message>
case studies with 90-50
</commit_message>
<xml_diff>
--- a/case_studies/base_case_50_5_dd/2050/technologies.xlsx
+++ b/case_studies/base_case_50_5_dd/2050/technologies.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\base_case_10_dd\2050\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\base_case_50_5_dd\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_FDB96DFE316C90107E524FD4235BDA1626C6999C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E884BE-FA78-4BCB-9E52-263751C08958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="1" r:id="rId1"/>
@@ -676,7 +676,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="3">
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3">
         <v>0</v>
@@ -685,55 +685,55 @@
         <v>0</v>
       </c>
       <c r="I2" s="3">
-        <v>114.1</v>
+        <v>0</v>
       </c>
       <c r="J2" s="3">
-        <v>462.87</v>
+        <v>0</v>
       </c>
       <c r="K2" s="3">
-        <v>99.04</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3">
-        <v>66.95</v>
+        <v>0</v>
       </c>
       <c r="M2" s="3">
-        <v>946.41</v>
+        <v>0</v>
       </c>
       <c r="N2" s="3">
-        <v>983.99</v>
+        <v>0</v>
       </c>
       <c r="O2" s="3">
         <v>0</v>
       </c>
       <c r="P2" s="3">
-        <v>370.48</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="3">
-        <v>416.03</v>
+        <v>0</v>
       </c>
       <c r="R2" s="3">
-        <v>36.799999999999997</v>
+        <v>0</v>
       </c>
       <c r="S2" s="3">
-        <v>22.37</v>
+        <v>0</v>
       </c>
       <c r="T2" s="3">
-        <v>181.05</v>
+        <v>0</v>
       </c>
       <c r="U2" s="3">
         <v>0</v>
       </c>
       <c r="V2" s="3">
-        <v>49.16</v>
+        <v>0</v>
       </c>
       <c r="W2" s="3">
-        <v>274.69</v>
+        <v>0</v>
       </c>
       <c r="X2" s="3">
-        <v>6.85</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="3">
-        <v>5784</v>
+        <v>0</v>
       </c>
       <c r="Z2" s="3">
         <v>0</v>
@@ -759,34 +759,34 @@
         <v>32</v>
       </c>
       <c r="B3" s="5">
-        <v>5.21</v>
+        <v>0</v>
       </c>
       <c r="C3" s="5">
         <v>0</v>
       </c>
       <c r="D3" s="5">
-        <v>45.66</v>
+        <v>0</v>
       </c>
       <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" s="5">
-        <v>1.44</v>
+        <v>0</v>
       </c>
       <c r="G3" s="5">
-        <v>8.08</v>
+        <v>0</v>
       </c>
       <c r="H3" s="5">
-        <v>3.55</v>
+        <v>0</v>
       </c>
       <c r="I3" s="5">
         <v>0</v>
       </c>
       <c r="J3" s="5">
-        <v>37.72</v>
+        <v>0</v>
       </c>
       <c r="K3" s="5">
-        <v>35.22</v>
+        <v>0</v>
       </c>
       <c r="L3" s="5">
         <v>0</v>
@@ -813,7 +813,7 @@
         <v>0</v>
       </c>
       <c r="T3" s="5">
-        <v>17.75</v>
+        <v>0</v>
       </c>
       <c r="U3" s="5">
         <v>0</v>
@@ -831,7 +831,7 @@
         <v>0</v>
       </c>
       <c r="Z3" s="5">
-        <v>48.42</v>
+        <v>0</v>
       </c>
       <c r="AA3" s="5">
         <v>0</v>
@@ -860,73 +860,73 @@
         <v>0</v>
       </c>
       <c r="D4" s="3">
-        <v>39.950000000000003</v>
+        <v>0</v>
       </c>
       <c r="E4" s="3">
         <v>0</v>
       </c>
       <c r="F4" s="3">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3">
-        <v>7.07</v>
+        <v>0</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
       </c>
       <c r="I4" s="3">
-        <v>177.04</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3">
-        <v>541.75</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3">
-        <v>20.3</v>
+        <v>0</v>
       </c>
       <c r="L4" s="3">
-        <v>313.55</v>
+        <v>0</v>
       </c>
       <c r="M4" s="3">
-        <v>666.6</v>
+        <v>0</v>
       </c>
       <c r="N4" s="3">
-        <v>666.6</v>
+        <v>0</v>
       </c>
       <c r="O4" s="3">
         <v>0</v>
       </c>
       <c r="P4" s="3">
-        <v>1217.3399999999999</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3">
-        <v>1252.6199999999999</v>
+        <v>0</v>
       </c>
       <c r="R4" s="3">
-        <v>254.91</v>
+        <v>0</v>
       </c>
       <c r="S4" s="3">
-        <v>43.32</v>
+        <v>0</v>
       </c>
       <c r="T4" s="3">
-        <v>490.59</v>
+        <v>0</v>
       </c>
       <c r="U4" s="3">
         <v>0</v>
       </c>
       <c r="V4" s="3">
-        <v>14.73</v>
+        <v>0</v>
       </c>
       <c r="W4" s="3">
-        <v>251.91</v>
+        <v>0</v>
       </c>
       <c r="X4" s="3">
-        <v>13.7</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
         <v>0</v>
       </c>
       <c r="Z4" s="3">
-        <v>27.91</v>
+        <v>0</v>
       </c>
       <c r="AA4" s="3">
         <v>0</v>
@@ -955,46 +955,46 @@
         <v>0</v>
       </c>
       <c r="D5" s="5">
-        <v>216.89</v>
+        <v>0</v>
       </c>
       <c r="E5" s="5">
         <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>2.96</v>
+        <v>0</v>
       </c>
       <c r="G5" s="5">
-        <v>38.39</v>
+        <v>0</v>
       </c>
       <c r="H5" s="5">
-        <v>0.56000000000000005</v>
+        <v>0</v>
       </c>
       <c r="I5" s="5">
-        <v>109.13</v>
+        <v>0</v>
       </c>
       <c r="J5" s="5">
-        <v>425.64</v>
+        <v>0</v>
       </c>
       <c r="K5" s="5">
-        <v>161.81</v>
+        <v>0</v>
       </c>
       <c r="L5" s="5">
-        <v>166.88</v>
+        <v>0</v>
       </c>
       <c r="M5" s="5">
-        <v>745.4</v>
+        <v>0</v>
       </c>
       <c r="N5" s="5">
-        <v>745.4</v>
+        <v>0</v>
       </c>
       <c r="O5" s="5">
         <v>0</v>
       </c>
       <c r="P5" s="5">
-        <v>440.9</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="5">
-        <v>440.9</v>
+        <v>0</v>
       </c>
       <c r="R5" s="5">
         <v>0</v>
@@ -1003,7 +1003,7 @@
         <v>0</v>
       </c>
       <c r="T5" s="5">
-        <v>276.01</v>
+        <v>0</v>
       </c>
       <c r="U5" s="5">
         <v>0</v>
@@ -1012,16 +1012,16 @@
         <v>0</v>
       </c>
       <c r="W5" s="5">
-        <v>369.14</v>
+        <v>0</v>
       </c>
       <c r="X5" s="5">
-        <v>13.7</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="5">
-        <v>19990</v>
+        <v>0</v>
       </c>
       <c r="Z5" s="5">
-        <v>204.22</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="5">
         <v>0</v>
@@ -1047,7 +1047,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="3">
-        <v>0.96</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3">
         <v>0</v>
@@ -1065,40 +1065,40 @@
         <v>0</v>
       </c>
       <c r="I6" s="3">
-        <v>64.790000000000006</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3">
-        <v>159.69999999999999</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3">
         <v>0</v>
       </c>
       <c r="L6" s="3">
-        <v>166.74</v>
+        <v>0</v>
       </c>
       <c r="M6" s="3">
-        <v>187.94</v>
+        <v>0</v>
       </c>
       <c r="N6" s="3">
-        <v>187.94</v>
+        <v>0</v>
       </c>
       <c r="O6" s="3">
         <v>0</v>
       </c>
       <c r="P6" s="3">
-        <v>526.65</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="3">
-        <v>526.65</v>
+        <v>0</v>
       </c>
       <c r="R6" s="3">
-        <v>55.31</v>
+        <v>0</v>
       </c>
       <c r="S6" s="3">
         <v>0</v>
       </c>
       <c r="T6" s="3">
-        <v>231.53</v>
+        <v>0</v>
       </c>
       <c r="U6" s="3">
         <v>0</v>
@@ -1107,10 +1107,10 @@
         <v>0</v>
       </c>
       <c r="W6" s="3">
-        <v>55.31</v>
+        <v>0</v>
       </c>
       <c r="X6" s="3">
-        <v>13.7</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="3">
         <v>0</v>
@@ -1160,10 +1160,10 @@
         <v>0</v>
       </c>
       <c r="I7" s="5">
-        <v>48.52</v>
+        <v>0</v>
       </c>
       <c r="J7" s="5">
-        <v>59.3</v>
+        <v>0</v>
       </c>
       <c r="K7" s="5">
         <v>0</v>
@@ -1181,28 +1181,28 @@
         <v>0</v>
       </c>
       <c r="P7" s="5">
-        <v>97.03</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="5">
         <v>0</v>
       </c>
       <c r="R7" s="5">
-        <v>18.48</v>
+        <v>0</v>
       </c>
       <c r="S7" s="5">
-        <v>15.14</v>
+        <v>0</v>
       </c>
       <c r="T7" s="5">
-        <v>48.52</v>
+        <v>0</v>
       </c>
       <c r="U7" s="5">
         <v>0</v>
       </c>
       <c r="V7" s="5">
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="W7" s="5">
-        <v>18.38</v>
+        <v>0</v>
       </c>
       <c r="X7" s="5">
         <v>0</v>
@@ -1255,55 +1255,55 @@
         <v>0</v>
       </c>
       <c r="I8" s="3">
-        <v>108.82</v>
+        <v>0</v>
       </c>
       <c r="J8" s="3">
-        <v>284.42</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3">
-        <v>46.55</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3">
-        <v>107.99</v>
+        <v>0</v>
       </c>
       <c r="M8" s="3">
-        <v>136.33000000000001</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3">
-        <v>136.33000000000001</v>
+        <v>0</v>
       </c>
       <c r="O8" s="3">
         <v>0</v>
       </c>
       <c r="P8" s="3">
-        <v>408.4</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3">
-        <v>492.95</v>
+        <v>0</v>
       </c>
       <c r="R8" s="3">
-        <v>130.06</v>
+        <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>73.62</v>
+        <v>0</v>
       </c>
       <c r="T8" s="3">
-        <v>216.81</v>
+        <v>0</v>
       </c>
       <c r="U8" s="3">
         <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>2.0499999999999998</v>
+        <v>0</v>
       </c>
       <c r="W8" s="3">
-        <v>311.61</v>
+        <v>0</v>
       </c>
       <c r="X8" s="3">
-        <v>13.7</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="3">
-        <v>19990</v>
+        <v>0</v>
       </c>
       <c r="Z8" s="3">
         <v>0</v>

</xml_diff>